<commit_message>
Publish full-run resumo por agente (2009–2010 BNDES)
Regenerate agent ranking Excel/CSV from the complete open-data
download (348,864 contracts, 72 agents) without requiring Streamlit.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_por_agente.xlsx
+++ b/output/resumo_por_agente.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,129 +441,1153 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BANCO SANTANDER BRASIL SA</t>
+          <t>BANCO DO BRASIL SA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>42113</v>
       </c>
       <c r="C2" t="n">
-        <v>302008.36</v>
+        <v>5813322583.31</v>
       </c>
       <c r="D2" t="n">
-        <v>2210450.08</v>
+        <v>42862815164.79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BANCO BRADESCO SA</t>
+          <t>ITAU UNIBANCO S.A.</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>56467</v>
       </c>
       <c r="C3" t="n">
-        <v>211466.62</v>
+        <v>4508481207.07</v>
       </c>
       <c r="D3" t="n">
-        <v>1658033.8</v>
+        <v>35542713355.21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL SA</t>
+          <t>BANCO BRADESCO S.A.</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>56957</v>
       </c>
       <c r="C4" t="n">
-        <v>187504.11</v>
+        <v>3962836137.45</v>
       </c>
       <c r="D4" t="n">
-        <v>1648196.56</v>
+        <v>31640455622.42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ITAU UNIBANCO SA</t>
+          <t>BANCO VOLKSWAGEN S.A.</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>50036</v>
       </c>
       <c r="C5" t="n">
-        <v>184992.67</v>
+        <v>1417954266.99</v>
       </c>
       <c r="D5" t="n">
-        <v>1496096.08</v>
+        <v>12087580442.84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
+          <t>BANCO SANTANDER (BRASIL) S.A.</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>13238</v>
       </c>
       <c r="C6" t="n">
-        <v>50114.58</v>
+        <v>1181981193.66</v>
       </c>
       <c r="D6" t="n">
-        <v>396720.98</v>
+        <v>9829504062.84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO SICREDI SA</t>
+          <t>BANCO MERCEDES-BENZ DO BRASIL S/A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>22681</v>
       </c>
       <c r="C7" t="n">
-        <v>27921.87</v>
+        <v>1108515246.59</v>
       </c>
       <c r="D7" t="n">
-        <v>263325.65</v>
+        <v>9493101007.049999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAIXA ECONOMICA FEDERAL</t>
+          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>8402</v>
       </c>
       <c r="C8" t="n">
-        <v>21311.25</v>
+        <v>1073343467.69</v>
       </c>
       <c r="D8" t="n">
-        <v>190057.65</v>
+        <v>7768708221.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO DO BRASIL SA - BANCOOB</t>
+          <t>BANCO SAFRA S A</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>12463</v>
+      </c>
+      <c r="C9" t="n">
+        <v>885746988.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7302263356</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BANCO VOTORANTIM S.A.</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4316</v>
+      </c>
+      <c r="C10" t="n">
+        <v>830916025.78</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6594730325.32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KIRTON BANK S.A. - BANCO MULTIPLO</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3130</v>
+      </c>
+      <c r="C11" t="n">
+        <v>423566822.19</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3568129160.61</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BANCO CATERPILLAR S.A.</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4783</v>
+      </c>
+      <c r="C12" t="n">
+        <v>419288448.44</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3483294379.69</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BANCO ABC BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C13" t="n">
+        <v>378470477.52</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3110969134.18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BANCO VOLVO (BRASIL) S.A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5818</v>
+      </c>
+      <c r="C14" t="n">
+        <v>326751159.13</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2703909991.84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CAIXA ECONOMICA FEDERAL</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5071</v>
+      </c>
+      <c r="C15" t="n">
+        <v>303357067.47</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2400673834.18</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICREDI S.A.</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>12554</v>
+      </c>
+      <c r="C16" t="n">
+        <v>295205730.45</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2153191448.35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A. - BDMG</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>631</v>
+      </c>
+      <c r="C17" t="n">
+        <v>244693215.62</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1781379447.84</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BADESUL DESENVOLVIMENTO S.A. - AGENCIA DE FOMENTO/RS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>968</v>
+      </c>
+      <c r="C18" t="n">
+        <v>241045387.88</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1757171113.73</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BANCO STELLANTIS S.A.</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4554</v>
+      </c>
+      <c r="C19" t="n">
+        <v>188321022.18</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1572006247.47</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DO RIO GRANDE DO SUL SA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3542</v>
+      </c>
+      <c r="C20" t="n">
+        <v>175613234.04</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1328013875.33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BANCO PINE S/A</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>145</v>
+      </c>
+      <c r="C21" t="n">
+        <v>159652368.36</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1141094301.74</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BANCO DE LAGE LANDEN BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1214</v>
+      </c>
+      <c r="C22" t="n">
+        <v>132195854.95</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1052390735.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DO ESPIRITO SANTO S/A</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5011</v>
+      </c>
+      <c r="C23" t="n">
+        <v>108313413.05</v>
+      </c>
+      <c r="D23" t="n">
+        <v>766406668.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BANCO MONEO S.A.</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1177</v>
+      </c>
+      <c r="C24" t="n">
+        <v>102707635.63</v>
+      </c>
+      <c r="D24" t="n">
+        <v>840075557.64</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO COM INTERACAO SOLIDARIA</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8118</v>
+      </c>
+      <c r="C25" t="n">
+        <v>97197667.26000001</v>
+      </c>
+      <c r="D25" t="n">
+        <v>750522203.35</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO E ECONOMIA COM INTERACAO</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>6909</v>
+      </c>
+      <c r="C26" t="n">
+        <v>89367857.13</v>
+      </c>
+      <c r="D26" t="n">
+        <v>685054153.28</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SAFRA LEASING S.A. ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C27" t="n">
+        <v>79726677.12</v>
+      </c>
+      <c r="D27" t="n">
+        <v>708185808.7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BANCO DA AMAZONIA SA / FINAM</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>41</v>
+      </c>
+      <c r="C28" t="n">
+        <v>78009100.55</v>
+      </c>
+      <c r="D28" t="n">
+        <v>547758578.9400001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BANCO CNH INDUSTRIAL CAPITAL S.A.</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1154</v>
+      </c>
+      <c r="C29" t="n">
+        <v>74943751.7</v>
+      </c>
+      <c r="D29" t="n">
+        <v>642248838.95</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BANCO ALFA DE INVESTIMENTO S.A.</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>337</v>
+      </c>
+      <c r="C30" t="n">
+        <v>70422205.70999999</v>
+      </c>
+      <c r="D30" t="n">
+        <v>572843332.9400001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICOOB S.A.</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>4244</v>
+      </c>
+      <c r="C31" t="n">
+        <v>61699291.98</v>
+      </c>
+      <c r="D31" t="n">
+        <v>462476854.88</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BANCO DAYCOVAL S.A.</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>408</v>
+      </c>
+      <c r="C32" t="n">
+        <v>60026314.73</v>
+      </c>
+      <c r="D32" t="n">
+        <v>486555126.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BANCO RODOBENS S.A.</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2380</v>
+      </c>
+      <c r="C33" t="n">
+        <v>56243108.57</v>
+      </c>
+      <c r="D33" t="n">
+        <v>482966606.87</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BRADESCO LEASING S.A. - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>844</v>
+      </c>
+      <c r="C34" t="n">
+        <v>54321791.01</v>
+      </c>
+      <c r="D34" t="n">
+        <v>455895941.94</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BANCO DO NORDESTE DO BRASIL SA / FINOR</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>752</v>
+      </c>
+      <c r="C35" t="n">
+        <v>48479935.33</v>
+      </c>
+      <c r="D35" t="n">
+        <v>323758674.79</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BANCO FIBRA SA</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>292</v>
+      </c>
+      <c r="C36" t="n">
+        <v>46721856.08</v>
+      </c>
+      <c r="D36" t="n">
+        <v>415528051.33</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BANCO CITIBANK S A</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>320</v>
+      </c>
+      <c r="C37" t="n">
+        <v>44928607.78</v>
+      </c>
+      <c r="D37" t="n">
+        <v>377359324.67</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BANCO GUANABARA S/A</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>807</v>
+      </c>
+      <c r="C38" t="n">
+        <v>36925603.12</v>
+      </c>
+      <c r="D38" t="n">
+        <v>324112553.99</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SCANIA BANCO S.A.</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>395</v>
+      </c>
+      <c r="C39" t="n">
+        <v>35104893.03</v>
+      </c>
+      <c r="D39" t="n">
+        <v>266832495.92</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BANCO JOHN DEERE S.A.</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>374</v>
+      </c>
+      <c r="C40" t="n">
+        <v>34464833.34</v>
+      </c>
+      <c r="D40" t="n">
+        <v>276501179.25</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FINANCEIRA ALFA S.A. CREDITO, FINANCIAMENTO E INVESTIME</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>275</v>
+      </c>
+      <c r="C41" t="n">
+        <v>32943362.39</v>
+      </c>
+      <c r="D41" t="n">
+        <v>290629108.58</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MERCEDES-BENZ LEASING DO BRASIL ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>910</v>
+      </c>
+      <c r="C42" t="n">
+        <v>32134027.26</v>
+      </c>
+      <c r="D42" t="n">
+        <v>288725718.63</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BANESTES SA BANCO DO ESTADO DO ESPIRITO SANTO</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>144</v>
+      </c>
+      <c r="C43" t="n">
+        <v>23686521.34</v>
+      </c>
+      <c r="D43" t="n">
+        <v>196120326.63</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DE SANTA CATARINA S.A. - B</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>104</v>
+      </c>
+      <c r="C44" t="n">
+        <v>20958523.95</v>
+      </c>
+      <c r="D44" t="n">
+        <v>174856984.5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BANCO RENDIMENTO S/A</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>84</v>
+      </c>
+      <c r="C45" t="n">
+        <v>18959696.36</v>
+      </c>
+      <c r="D45" t="n">
+        <v>157526255.82</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DESENVOLVE SP AGENCIA DE FOMENTO DO ESTADO DE SAO PAULO</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>214</v>
+      </c>
+      <c r="C46" t="n">
+        <v>18225304.83</v>
+      </c>
+      <c r="D46" t="n">
+        <v>153868993.21</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BANCO RIBEIRAO PRETO S/A</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>76</v>
+      </c>
+      <c r="C47" t="n">
+        <v>17691750.56</v>
+      </c>
+      <c r="D47" t="n">
+        <v>144336280.78</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BANCO VOITER SA</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>95</v>
+      </c>
+      <c r="C48" t="n">
+        <v>15266010.92</v>
+      </c>
+      <c r="D48" t="n">
+        <v>122064376.97</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BANCO ITAULEASING S.A.</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>271</v>
+      </c>
+      <c r="C49" t="n">
+        <v>13974268.19</v>
+      </c>
+      <c r="D49" t="n">
+        <v>114961488.29</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BANCO BMG S.A</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>232</v>
+      </c>
+      <c r="C50" t="n">
+        <v>13571635.88</v>
+      </c>
+      <c r="D50" t="n">
+        <v>118285729.55</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO AMAZONAS S.A. - AFEAM</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>13</v>
+      </c>
+      <c r="C51" t="n">
+        <v>11958337.31</v>
+      </c>
+      <c r="D51" t="n">
+        <v>87412128.33</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BANCO RABOBANK INTERNATIONAL BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>39</v>
+      </c>
+      <c r="C52" t="n">
+        <v>11562602.07</v>
+      </c>
+      <c r="D52" t="n">
+        <v>84316529.13</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BRB BANCO DE BRASILIA SA</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>23</v>
+      </c>
+      <c r="C53" t="n">
+        <v>10080141.04</v>
+      </c>
+      <c r="D53" t="n">
+        <v>79670064.89</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BANCO INDUSTRIAL DO BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>107</v>
+      </c>
+      <c r="C54" t="n">
+        <v>9869376.43</v>
+      </c>
+      <c r="D54" t="n">
+        <v>85730081.84999999</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DIBENS LEASING S/A - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>112</v>
+      </c>
+      <c r="C55" t="n">
+        <v>9846881.76</v>
+      </c>
+      <c r="D55" t="n">
+        <v>88417485.23</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BANCO J. SAFRA S.A</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>85</v>
+      </c>
+      <c r="C56" t="n">
+        <v>6699793.46</v>
+      </c>
+      <c r="D56" t="n">
+        <v>64192863.86</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO RIO DE JANEIRO S. A.</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>18</v>
+      </c>
+      <c r="C57" t="n">
+        <v>6549074.48</v>
+      </c>
+      <c r="D57" t="n">
+        <v>52693631.75</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BANCO SOFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>62</v>
+      </c>
+      <c r="C58" t="n">
+        <v>6385827.35</v>
+      </c>
+      <c r="D58" t="n">
+        <v>59596246.13</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DE SERGIPE S/A</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>22</v>
+      </c>
+      <c r="C59" t="n">
+        <v>5272502.19</v>
+      </c>
+      <c r="D59" t="n">
+        <v>37479426.25</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BANCO BTG PACTUAL S.A.</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>14</v>
+      </c>
+      <c r="C60" t="n">
+        <v>5034002.96</v>
+      </c>
+      <c r="D60" t="n">
+        <v>43283234.7</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BANCO TRIANGULO S/A</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>43</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4635118.33</v>
+      </c>
+      <c r="D61" t="n">
+        <v>37422550.97</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DESENBAHIA-AGENCIA DE FOMENTO DO ESTADO DA BAHIA S/A</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>29</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4554879.66</v>
+      </c>
+      <c r="D62" t="n">
+        <v>35009843.09</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BANCO CREFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>25</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3165854.9</v>
+      </c>
+      <c r="D63" t="n">
+        <v>30705663.36</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BANCO BV S.A.</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>40</v>
+      </c>
+      <c r="C64" t="n">
+        <v>2905151.1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>25172134.8</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BMG LEASING SA ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>41</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2542204.06</v>
+      </c>
+      <c r="D65" t="n">
+        <v>22147542.09</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BB.LEASING S.A.ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>17</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1140244.25</v>
+      </c>
+      <c r="D66" t="n">
+        <v>8062621.86</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BRKB DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS S.A</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="n">
-        <v>6937.5</v>
-      </c>
-      <c r="D9" t="n">
-        <v>60106.74</v>
+      <c r="C67" t="n">
+        <v>551250</v>
+      </c>
+      <c r="D67" t="n">
+        <v>5067716.74</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BANCO RANDON SA</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="n">
+        <v>482574.84</v>
+      </c>
+      <c r="D68" t="n">
+        <v>3592216.32</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DIRECAO S A CREDITO FINANCIAMENTO E INVESTIMENTO</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>6</v>
+      </c>
+      <c r="C69" t="n">
+        <v>285646.61</v>
+      </c>
+      <c r="D69" t="n">
+        <v>2534597.25</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO PARANA S.A.</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="n">
+        <v>195695.52</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1430643.05</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO TOCANTINS S.A.</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" t="n">
+        <v>189985.5</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1395991.35</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BANCO PORTO REAL DE INVESTIMENTOS S/A</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>94720.14999999999</v>
+      </c>
+      <c r="D72" t="n">
+        <v>823495.75</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BONCRED FINANCEIRA S.A. - CREDITO, FINANCIAMENTO E INVE</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" t="n">
+        <v>37990.35</v>
+      </c>
+      <c r="D73" t="n">
+        <v>332347.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish full-run detailed ContAgil flows for 2009–2010
Regenerate fluxos_completos_final.xlsx and agent ranking from the full
BNDES open dataset (348,864 contracts, 22.15M parcels) using compound
monthly rates and detailed ContAgil columns. Add 1k-row sample Excel.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_por_agente.xlsx
+++ b/output/resumo_por_agente.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,129 +441,1153 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BANCO SANTANDER BRASIL SA</t>
+          <t>BANCO DO BRASIL SA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>42113</v>
       </c>
       <c r="C2" t="n">
-        <v>278419.45</v>
+        <v>5341100463.42</v>
       </c>
       <c r="D2" t="n">
-        <v>1823870.05</v>
+        <v>35208245592.46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BANCO BRADESCO SA</t>
+          <t>ITAU UNIBANCO S.A.</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>56467</v>
       </c>
       <c r="C3" t="n">
-        <v>194561.72</v>
+        <v>4135945773.13</v>
       </c>
       <c r="D3" t="n">
-        <v>1359984.44</v>
+        <v>29051608594.83</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL SA</t>
+          <t>BANCO BRADESCO S.A.</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>56957</v>
       </c>
       <c r="C4" t="n">
-        <v>171859.57</v>
+        <v>3633054899.21</v>
       </c>
       <c r="D4" t="n">
-        <v>1338244.62</v>
+        <v>25832400897.94</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ITAU UNIBANCO SA</t>
+          <t>BANCO VOLKSWAGEN S.A.</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>50036</v>
       </c>
       <c r="C5" t="n">
-        <v>169963.48</v>
+        <v>1296591623.5</v>
       </c>
       <c r="D5" t="n">
-        <v>1223393.4</v>
+        <v>9812854459.42</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
+          <t>BANCO SANTANDER (BRASIL) S.A.</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>13238</v>
       </c>
       <c r="C6" t="n">
-        <v>45846.49</v>
+        <v>1084182486.84</v>
       </c>
       <c r="D6" t="n">
-        <v>323583.93</v>
+        <v>8012360384.58</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO SICREDI SA</t>
+          <t>BANCO MERCEDES-BENZ DO BRASIL S/A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>22681</v>
       </c>
       <c r="C7" t="n">
-        <v>25504.66</v>
+        <v>1014242948.99</v>
       </c>
       <c r="D7" t="n">
-        <v>212271.05</v>
+        <v>7709153253.87</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAIXA ECONOMICA FEDERAL</t>
+          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>8402</v>
       </c>
       <c r="C8" t="n">
-        <v>19432.36</v>
+        <v>984715144.34</v>
       </c>
       <c r="D8" t="n">
-        <v>153424.44</v>
+        <v>6376457745.64</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO DO BRASIL SA - BANCOOB</t>
+          <t>BANCO SAFRA S A</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>12463</v>
+      </c>
+      <c r="C9" t="n">
+        <v>809780070.38</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5937528733.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BANCO VOTORANTIM S.A.</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4316</v>
+      </c>
+      <c r="C10" t="n">
+        <v>761998368.98</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5383157976.22</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KIRTON BANK S.A. - BANCO MULTIPLO</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3130</v>
+      </c>
+      <c r="C11" t="n">
+        <v>388257303.01</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2904823948.16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BANCO CATERPILLAR S.A.</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4783</v>
+      </c>
+      <c r="C12" t="n">
+        <v>386132093.14</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2850987864.29</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BANCO ABC BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C13" t="n">
+        <v>346296018.75</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2530631131.65</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BANCO VOLVO (BRASIL) S.A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5818</v>
+      </c>
+      <c r="C14" t="n">
+        <v>299018659.68</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2200587451.92</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CAIXA ECONOMICA FEDERAL</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5071</v>
+      </c>
+      <c r="C15" t="n">
+        <v>278237123.01</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1962321129.02</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICREDI S.A.</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>12554</v>
+      </c>
+      <c r="C16" t="n">
+        <v>273580750.27</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1784685804.3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A. - BDMG</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>631</v>
+      </c>
+      <c r="C17" t="n">
+        <v>225065011.59</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1465800283.67</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BADESUL DESENVOLVIMENTO S.A. - AGENCIA DE FOMENTO/RS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>968</v>
+      </c>
+      <c r="C18" t="n">
+        <v>221513408.22</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1444153440.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BANCO STELLANTIS S.A.</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4554</v>
+      </c>
+      <c r="C19" t="n">
+        <v>172291920.22</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1278378516.46</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DO RIO GRANDE DO SUL SA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3542</v>
+      </c>
+      <c r="C20" t="n">
+        <v>162181525.97</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1094592486.46</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BANCO PINE S/A</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>145</v>
+      </c>
+      <c r="C21" t="n">
+        <v>146127004.91</v>
+      </c>
+      <c r="D21" t="n">
+        <v>935259840.27</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BANCO DE LAGE LANDEN BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1214</v>
+      </c>
+      <c r="C22" t="n">
+        <v>121523832.93</v>
+      </c>
+      <c r="D22" t="n">
+        <v>862047552.05</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DO ESPIRITO SANTO S/A</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5011</v>
+      </c>
+      <c r="C23" t="n">
+        <v>100638150.52</v>
+      </c>
+      <c r="D23" t="n">
+        <v>637898381.23</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BANCO MONEO S.A.</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1177</v>
+      </c>
+      <c r="C24" t="n">
+        <v>93618588.05</v>
+      </c>
+      <c r="D24" t="n">
+        <v>681036876.59</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO COM INTERACAO SOLIDARIA</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8118</v>
+      </c>
+      <c r="C25" t="n">
+        <v>90357570.64</v>
+      </c>
+      <c r="D25" t="n">
+        <v>621790047.88</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO E ECONOMIA COM INTERACAO</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>6909</v>
+      </c>
+      <c r="C26" t="n">
+        <v>83013175.06999999</v>
+      </c>
+      <c r="D26" t="n">
+        <v>567400080</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SAFRA LEASING S.A. ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C27" t="n">
+        <v>72939004.75</v>
+      </c>
+      <c r="D27" t="n">
+        <v>573700481.28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BANCO DA AMAZONIA SA / FINAM</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>41</v>
+      </c>
+      <c r="C28" t="n">
+        <v>71672467.09</v>
+      </c>
+      <c r="D28" t="n">
+        <v>451055248.39</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BANCO CNH INDUSTRIAL CAPITAL S.A.</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1154</v>
+      </c>
+      <c r="C29" t="n">
+        <v>68871369.95999999</v>
+      </c>
+      <c r="D29" t="n">
+        <v>523710532.19</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BANCO ALFA DE INVESTIMENTO S.A.</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>337</v>
+      </c>
+      <c r="C30" t="n">
+        <v>64836074.46</v>
+      </c>
+      <c r="D30" t="n">
+        <v>469230760.72</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICOOB S.A.</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>4244</v>
+      </c>
+      <c r="C31" t="n">
+        <v>56960724.06</v>
+      </c>
+      <c r="D31" t="n">
+        <v>381230137.48</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BANCO DAYCOVAL S.A.</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>408</v>
+      </c>
+      <c r="C32" t="n">
+        <v>54878861.17</v>
+      </c>
+      <c r="D32" t="n">
+        <v>395748633.17</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BANCO RODOBENS S.A.</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2380</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51294982.03</v>
+      </c>
+      <c r="D33" t="n">
+        <v>390820706.17</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BRADESCO LEASING S.A. - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>844</v>
+      </c>
+      <c r="C34" t="n">
+        <v>49858498.58</v>
+      </c>
+      <c r="D34" t="n">
+        <v>371596066.7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BANCO DO NORDESTE DO BRASIL SA / FINOR</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>752</v>
+      </c>
+      <c r="C35" t="n">
+        <v>44547311.64</v>
+      </c>
+      <c r="D35" t="n">
+        <v>267539533.05</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BANCO FIBRA SA</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>292</v>
+      </c>
+      <c r="C36" t="n">
+        <v>42638582.93</v>
+      </c>
+      <c r="D36" t="n">
+        <v>335805620.57</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BANCO CITIBANK S A</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>320</v>
+      </c>
+      <c r="C37" t="n">
+        <v>40990391.88</v>
+      </c>
+      <c r="D37" t="n">
+        <v>305802670.91</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BANCO GUANABARA S/A</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>807</v>
+      </c>
+      <c r="C38" t="n">
+        <v>33621577.15</v>
+      </c>
+      <c r="D38" t="n">
+        <v>261562470.09</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SCANIA BANCO S.A.</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>395</v>
+      </c>
+      <c r="C39" t="n">
+        <v>31925061.26</v>
+      </c>
+      <c r="D39" t="n">
+        <v>216897470.57</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BANCO JOHN DEERE S.A.</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>374</v>
+      </c>
+      <c r="C40" t="n">
+        <v>31572895.34</v>
+      </c>
+      <c r="D40" t="n">
+        <v>225405811.36</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FINANCEIRA ALFA S.A. CREDITO, FINANCIAMENTO E INVESTIME</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>275</v>
+      </c>
+      <c r="C41" t="n">
+        <v>30442890.41</v>
+      </c>
+      <c r="D41" t="n">
+        <v>237979217.69</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MERCEDES-BENZ LEASING DO BRASIL ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>910</v>
+      </c>
+      <c r="C42" t="n">
+        <v>29331080.64</v>
+      </c>
+      <c r="D42" t="n">
+        <v>233218176.59</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BANESTES SA BANCO DO ESTADO DO ESPIRITO SANTO</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>144</v>
+      </c>
+      <c r="C43" t="n">
+        <v>21782951.19</v>
+      </c>
+      <c r="D43" t="n">
+        <v>160301767.45</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DE SANTA CATARINA S.A. - B</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>104</v>
+      </c>
+      <c r="C44" t="n">
+        <v>19116806.88</v>
+      </c>
+      <c r="D44" t="n">
+        <v>141607450.19</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BANCO RENDIMENTO S/A</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>84</v>
+      </c>
+      <c r="C45" t="n">
+        <v>17390467.3</v>
+      </c>
+      <c r="D45" t="n">
+        <v>128352643.17</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DESENVOLVE SP AGENCIA DE FOMENTO DO ESTADO DE SAO PAULO</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>214</v>
+      </c>
+      <c r="C46" t="n">
+        <v>16734761.99</v>
+      </c>
+      <c r="D46" t="n">
+        <v>125469467.36</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BANCO RIBEIRAO PRETO S/A</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>76</v>
+      </c>
+      <c r="C47" t="n">
+        <v>16278109.7</v>
+      </c>
+      <c r="D47" t="n">
+        <v>118219701.91</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BANCO VOITER SA</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>95</v>
+      </c>
+      <c r="C48" t="n">
+        <v>14018314.94</v>
+      </c>
+      <c r="D48" t="n">
+        <v>100096659.71</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BANCO ITAULEASING S.A.</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>271</v>
+      </c>
+      <c r="C49" t="n">
+        <v>12785896.61</v>
+      </c>
+      <c r="D49" t="n">
+        <v>93564666.53</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BANCO BMG S.A</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>232</v>
+      </c>
+      <c r="C50" t="n">
+        <v>12405399.05</v>
+      </c>
+      <c r="D50" t="n">
+        <v>95860932.40000001</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO AMAZONAS S.A. - AFEAM</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>13</v>
+      </c>
+      <c r="C51" t="n">
+        <v>10963860.48</v>
+      </c>
+      <c r="D51" t="n">
+        <v>71657522.76000001</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BANCO RABOBANK INTERNATIONAL BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>39</v>
+      </c>
+      <c r="C52" t="n">
+        <v>10641060.28</v>
+      </c>
+      <c r="D52" t="n">
+        <v>69436604.48999999</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BRB BANCO DE BRASILIA SA</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>23</v>
+      </c>
+      <c r="C53" t="n">
+        <v>9241117.17</v>
+      </c>
+      <c r="D53" t="n">
+        <v>65021365.19</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BANCO INDUSTRIAL DO BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>107</v>
+      </c>
+      <c r="C54" t="n">
+        <v>9014630.560000001</v>
+      </c>
+      <c r="D54" t="n">
+        <v>69439507.62</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DIBENS LEASING S/A - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>112</v>
+      </c>
+      <c r="C55" t="n">
+        <v>8975145.720000001</v>
+      </c>
+      <c r="D55" t="n">
+        <v>71316425.16</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BANCO J. SAFRA S.A</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>85</v>
+      </c>
+      <c r="C56" t="n">
+        <v>6205254.78</v>
+      </c>
+      <c r="D56" t="n">
+        <v>52406955.32</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO RIO DE JANEIRO S. A.</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>18</v>
+      </c>
+      <c r="C57" t="n">
+        <v>5987175.05</v>
+      </c>
+      <c r="D57" t="n">
+        <v>42889050.07</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BANCO SOFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>62</v>
+      </c>
+      <c r="C58" t="n">
+        <v>5818096.47</v>
+      </c>
+      <c r="D58" t="n">
+        <v>47965406.03</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DE SERGIPE S/A</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>22</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4830549.81</v>
+      </c>
+      <c r="D59" t="n">
+        <v>30767927.25</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BANCO BTG PACTUAL S.A.</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>14</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4535918.69</v>
+      </c>
+      <c r="D60" t="n">
+        <v>34588526.63</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BANCO TRIANGULO S/A</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>43</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4233489.4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>30440752.43</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DESENBAHIA-AGENCIA DE FOMENTO DO ESTADO DA BAHIA S/A</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>29</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4182391.48</v>
+      </c>
+      <c r="D62" t="n">
+        <v>28686558.04</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BANCO CREFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>25</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2893966.57</v>
+      </c>
+      <c r="D63" t="n">
+        <v>24728075.43</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BANCO BV S.A.</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>40</v>
+      </c>
+      <c r="C64" t="n">
+        <v>2657290.88</v>
+      </c>
+      <c r="D64" t="n">
+        <v>20411521.36</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BMG LEASING SA ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>41</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2316504.14</v>
+      </c>
+      <c r="D65" t="n">
+        <v>17893656.29</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BB.LEASING S.A.ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>17</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1046753.96</v>
+      </c>
+      <c r="D66" t="n">
+        <v>6627608.41</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BRKB DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS S.A</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="n">
-        <v>6319.76</v>
-      </c>
-      <c r="D9" t="n">
-        <v>48575.92</v>
+      <c r="C67" t="n">
+        <v>500578.12</v>
+      </c>
+      <c r="D67" t="n">
+        <v>4067969.31</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BANCO RANDON SA</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="n">
+        <v>437755.41</v>
+      </c>
+      <c r="D68" t="n">
+        <v>2916177.36</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DIRECAO S A CREDITO FINANCIAMENTO E INVESTIMENTO</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>6</v>
+      </c>
+      <c r="C69" t="n">
+        <v>262156.21</v>
+      </c>
+      <c r="D69" t="n">
+        <v>2060152.92</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO PARANA S.A.</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="n">
+        <v>179800.31</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1176942.54</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO TOCANTINS S.A.</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" t="n">
+        <v>172883.32</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1137355.23</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BANCO PORTO REAL DE INVESTIMENTOS S/A</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>86880.42</v>
+      </c>
+      <c r="D72" t="n">
+        <v>669990.29</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BONCRED FINANCEIRA S.A. - CREDITO, FINANCIAMENTO E INVE</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" t="n">
+        <v>34604.71</v>
+      </c>
+      <c r="D73" t="n">
+        <v>268062.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza saídas com impacto fiscal via fatores SELIC Bacen.
Run completo 2009–2010: 348.864 contratos, 22.151.051 parcelas,
subsídio R$ 23,45 bi, impacto fiscal 2026 R$ 90,17 bi (72 agentes).

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_por_agente.xlsx
+++ b/output/resumo_por_agente.xlsx
@@ -451,7 +451,7 @@
         <v>5341100463.42</v>
       </c>
       <c r="D2" t="n">
-        <v>35208245592.46</v>
+        <v>19597821728.37</v>
       </c>
     </row>
     <row r="3">
@@ -467,7 +467,7 @@
         <v>4135945773.13</v>
       </c>
       <c r="D3" t="n">
-        <v>29051608594.83</v>
+        <v>15923837468.33</v>
       </c>
     </row>
     <row r="4">
@@ -483,7 +483,7 @@
         <v>3633054899.21</v>
       </c>
       <c r="D4" t="n">
-        <v>25832400897.94</v>
+        <v>14119377366.5</v>
       </c>
     </row>
     <row r="5">
@@ -499,7 +499,7 @@
         <v>1296591623.5</v>
       </c>
       <c r="D5" t="n">
-        <v>9812854459.42</v>
+        <v>5277080294.74</v>
       </c>
     </row>
     <row r="6">
@@ -515,7 +515,7 @@
         <v>1084182486.84</v>
       </c>
       <c r="D6" t="n">
-        <v>8012360384.58</v>
+        <v>4336268488.45</v>
       </c>
     </row>
     <row r="7">
@@ -531,7 +531,7 @@
         <v>1014242948.99</v>
       </c>
       <c r="D7" t="n">
-        <v>7709153253.87</v>
+        <v>4139189948.1</v>
       </c>
     </row>
     <row r="8">
@@ -547,7 +547,7 @@
         <v>984715144.34</v>
       </c>
       <c r="D8" t="n">
-        <v>6376457745.64</v>
+        <v>3566608966.73</v>
       </c>
     </row>
     <row r="9">
@@ -563,7 +563,7 @@
         <v>809780070.38</v>
       </c>
       <c r="D9" t="n">
-        <v>5937528733.1</v>
+        <v>3223796673.8</v>
       </c>
     </row>
     <row r="10">
@@ -579,7 +579,7 @@
         <v>761998368.98</v>
       </c>
       <c r="D10" t="n">
-        <v>5383157976.22</v>
+        <v>2950403055.02</v>
       </c>
     </row>
     <row r="11">
@@ -595,7 +595,7 @@
         <v>388257303.01</v>
       </c>
       <c r="D11" t="n">
-        <v>2904823948.16</v>
+        <v>1567802005.02</v>
       </c>
     </row>
     <row r="12">
@@ -611,7 +611,7 @@
         <v>386132093.14</v>
       </c>
       <c r="D12" t="n">
-        <v>2850987864.29</v>
+        <v>1541249391.65</v>
       </c>
     </row>
     <row r="13">
@@ -627,7 +627,7 @@
         <v>346296018.75</v>
       </c>
       <c r="D13" t="n">
-        <v>2530631131.65</v>
+        <v>1379273734.19</v>
       </c>
     </row>
     <row r="14">
@@ -643,7 +643,7 @@
         <v>299018659.68</v>
       </c>
       <c r="D14" t="n">
-        <v>2200587451.92</v>
+        <v>1193206737.85</v>
       </c>
     </row>
     <row r="15">
@@ -659,7 +659,7 @@
         <v>278237123.01</v>
       </c>
       <c r="D15" t="n">
-        <v>1962321129.02</v>
+        <v>1076153191.28</v>
       </c>
     </row>
     <row r="16">
@@ -675,7 +675,7 @@
         <v>273580750.27</v>
       </c>
       <c r="D16" t="n">
-        <v>1784685804.3</v>
+        <v>995660597.6</v>
       </c>
     </row>
     <row r="17">
@@ -691,7 +691,7 @@
         <v>225065011.59</v>
       </c>
       <c r="D17" t="n">
-        <v>1465800283.67</v>
+        <v>818180193.39</v>
       </c>
     </row>
     <row r="18">
@@ -707,7 +707,7 @@
         <v>221513408.22</v>
       </c>
       <c r="D18" t="n">
-        <v>1444153440.3</v>
+        <v>806112134.36</v>
       </c>
     </row>
     <row r="19">
@@ -723,7 +723,7 @@
         <v>172291920.22</v>
       </c>
       <c r="D19" t="n">
-        <v>1278378516.46</v>
+        <v>691514825.4299999</v>
       </c>
     </row>
     <row r="20">
@@ -739,7 +739,7 @@
         <v>162181525.97</v>
       </c>
       <c r="D20" t="n">
-        <v>1094592486.46</v>
+        <v>604911178.84</v>
       </c>
     </row>
     <row r="21">
@@ -755,7 +755,7 @@
         <v>146127004.91</v>
       </c>
       <c r="D21" t="n">
-        <v>935259840.27</v>
+        <v>525557110.71</v>
       </c>
     </row>
     <row r="22">
@@ -771,7 +771,7 @@
         <v>121523832.93</v>
       </c>
       <c r="D22" t="n">
-        <v>862047552.05</v>
+        <v>472313855.71</v>
       </c>
     </row>
     <row r="23">
@@ -787,7 +787,7 @@
         <v>100638150.52</v>
       </c>
       <c r="D23" t="n">
-        <v>637898381.23</v>
+        <v>358706638.27</v>
       </c>
     </row>
     <row r="24">
@@ -803,7 +803,7 @@
         <v>93618588.05</v>
       </c>
       <c r="D24" t="n">
-        <v>681036876.59</v>
+        <v>369989164.54</v>
       </c>
     </row>
     <row r="25">
@@ -819,7 +819,7 @@
         <v>90357570.64</v>
       </c>
       <c r="D25" t="n">
-        <v>621790047.88</v>
+        <v>341658621.51</v>
       </c>
     </row>
     <row r="26">
@@ -835,7 +835,7 @@
         <v>83013175.06999999</v>
       </c>
       <c r="D26" t="n">
-        <v>567400080</v>
+        <v>312515372.51</v>
       </c>
     </row>
     <row r="27">
@@ -851,7 +851,7 @@
         <v>72939004.75</v>
       </c>
       <c r="D27" t="n">
-        <v>573700481.28</v>
+        <v>305317231.47</v>
       </c>
     </row>
     <row r="28">
@@ -867,7 +867,7 @@
         <v>71672467.09</v>
       </c>
       <c r="D28" t="n">
-        <v>451055248.39</v>
+        <v>254060477.57</v>
       </c>
     </row>
     <row r="29">
@@ -883,7 +883,7 @@
         <v>68871369.95999999</v>
       </c>
       <c r="D29" t="n">
-        <v>523710532.19</v>
+        <v>281140346.73</v>
       </c>
     </row>
     <row r="30">
@@ -899,7 +899,7 @@
         <v>64836074.46</v>
       </c>
       <c r="D30" t="n">
-        <v>469230760.72</v>
+        <v>254967230.65</v>
       </c>
     </row>
     <row r="31">
@@ -915,7 +915,7 @@
         <v>56960724.06</v>
       </c>
       <c r="D31" t="n">
-        <v>381230137.48</v>
+        <v>211179595.15</v>
       </c>
     </row>
     <row r="32">
@@ -931,7 +931,7 @@
         <v>54878861.17</v>
       </c>
       <c r="D32" t="n">
-        <v>395748633.17</v>
+        <v>216586813.82</v>
       </c>
     </row>
     <row r="33">
@@ -947,7 +947,7 @@
         <v>51294982.03</v>
       </c>
       <c r="D33" t="n">
-        <v>390820706.17</v>
+        <v>209780558.11</v>
       </c>
     </row>
     <row r="34">
@@ -963,7 +963,7 @@
         <v>49858498.58</v>
       </c>
       <c r="D34" t="n">
-        <v>371596066.7</v>
+        <v>200444716.76</v>
       </c>
     </row>
     <row r="35">
@@ -979,7 +979,7 @@
         <v>44547311.64</v>
       </c>
       <c r="D35" t="n">
-        <v>267539533.05</v>
+        <v>152823706.02</v>
       </c>
     </row>
     <row r="36">
@@ -995,7 +995,7 @@
         <v>42638582.93</v>
       </c>
       <c r="D36" t="n">
-        <v>335805620.57</v>
+        <v>184257031.17</v>
       </c>
     </row>
     <row r="37">
@@ -1011,7 +1011,7 @@
         <v>40990391.88</v>
       </c>
       <c r="D37" t="n">
-        <v>305802670.91</v>
+        <v>165148849.21</v>
       </c>
     </row>
     <row r="38">
@@ -1027,7 +1027,7 @@
         <v>33621577.15</v>
       </c>
       <c r="D38" t="n">
-        <v>261562470.09</v>
+        <v>139575814.07</v>
       </c>
     </row>
     <row r="39">
@@ -1043,7 +1043,7 @@
         <v>31925061.26</v>
       </c>
       <c r="D39" t="n">
-        <v>216897470.57</v>
+        <v>120482812</v>
       </c>
     </row>
     <row r="40">
@@ -1059,7 +1059,7 @@
         <v>31572895.34</v>
       </c>
       <c r="D40" t="n">
-        <v>225405811.36</v>
+        <v>123057580.26</v>
       </c>
     </row>
     <row r="41">
@@ -1075,7 +1075,7 @@
         <v>30442890.41</v>
       </c>
       <c r="D41" t="n">
-        <v>237979217.69</v>
+        <v>126678129.32</v>
       </c>
     </row>
     <row r="42">
@@ -1091,7 +1091,7 @@
         <v>29331080.64</v>
       </c>
       <c r="D42" t="n">
-        <v>233218176.59</v>
+        <v>123675700.61</v>
       </c>
     </row>
     <row r="43">
@@ -1107,7 +1107,7 @@
         <v>21782951.19</v>
       </c>
       <c r="D43" t="n">
-        <v>160301767.45</v>
+        <v>86781865.09</v>
       </c>
     </row>
     <row r="44">
@@ -1123,7 +1123,7 @@
         <v>19116806.88</v>
       </c>
       <c r="D44" t="n">
-        <v>141607450.19</v>
+        <v>76538397.3</v>
       </c>
     </row>
     <row r="45">
@@ -1139,7 +1139,7 @@
         <v>17390467.3</v>
       </c>
       <c r="D45" t="n">
-        <v>128352643.17</v>
+        <v>69425385.92</v>
       </c>
     </row>
     <row r="46">
@@ -1155,7 +1155,7 @@
         <v>16734761.99</v>
       </c>
       <c r="D46" t="n">
-        <v>125469467.36</v>
+        <v>67710429.48</v>
       </c>
     </row>
     <row r="47">
@@ -1171,7 +1171,7 @@
         <v>16278109.7</v>
       </c>
       <c r="D47" t="n">
-        <v>118219701.91</v>
+        <v>67531614.01000001</v>
       </c>
     </row>
     <row r="48">
@@ -1187,7 +1187,7 @@
         <v>14018314.94</v>
       </c>
       <c r="D48" t="n">
-        <v>100096659.71</v>
+        <v>59508259.46</v>
       </c>
     </row>
     <row r="49">
@@ -1203,7 +1203,7 @@
         <v>12785896.61</v>
       </c>
       <c r="D49" t="n">
-        <v>93564666.53</v>
+        <v>50840421.2</v>
       </c>
     </row>
     <row r="50">
@@ -1219,7 +1219,7 @@
         <v>12405399.05</v>
       </c>
       <c r="D50" t="n">
-        <v>95860932.40000001</v>
+        <v>51292819.56</v>
       </c>
     </row>
     <row r="51">
@@ -1235,7 +1235,7 @@
         <v>10963860.48</v>
       </c>
       <c r="D51" t="n">
-        <v>71657522.76000001</v>
+        <v>39939343.23</v>
       </c>
     </row>
     <row r="52">
@@ -1251,7 +1251,7 @@
         <v>10641060.28</v>
       </c>
       <c r="D52" t="n">
-        <v>69436604.48999999</v>
+        <v>38821967.01</v>
       </c>
     </row>
     <row r="53">
@@ -1267,7 +1267,7 @@
         <v>9241117.17</v>
       </c>
       <c r="D53" t="n">
-        <v>65021365.19</v>
+        <v>35587428.92</v>
       </c>
     </row>
     <row r="54">
@@ -1283,7 +1283,7 @@
         <v>9014630.560000001</v>
       </c>
       <c r="D54" t="n">
-        <v>69439507.62</v>
+        <v>37182978.3</v>
       </c>
     </row>
     <row r="55">
@@ -1299,7 +1299,7 @@
         <v>8975145.720000001</v>
       </c>
       <c r="D55" t="n">
-        <v>71316425.16</v>
+        <v>37825163.82</v>
       </c>
     </row>
     <row r="56">
@@ -1315,7 +1315,7 @@
         <v>6205254.78</v>
       </c>
       <c r="D56" t="n">
-        <v>52406955.32</v>
+        <v>27290454.88</v>
       </c>
     </row>
     <row r="57">
@@ -1331,7 +1331,7 @@
         <v>5987175.05</v>
       </c>
       <c r="D57" t="n">
-        <v>42889050.07</v>
+        <v>23447385.91</v>
       </c>
     </row>
     <row r="58">
@@ -1347,7 +1347,7 @@
         <v>5818096.47</v>
       </c>
       <c r="D58" t="n">
-        <v>47965406.03</v>
+        <v>26372033.74</v>
       </c>
     </row>
     <row r="59">
@@ -1363,7 +1363,7 @@
         <v>4830549.81</v>
       </c>
       <c r="D59" t="n">
-        <v>30767927.25</v>
+        <v>17305379.07</v>
       </c>
     </row>
     <row r="60">
@@ -1379,7 +1379,7 @@
         <v>4535918.69</v>
       </c>
       <c r="D60" t="n">
-        <v>34588526.63</v>
+        <v>18585870.67</v>
       </c>
     </row>
     <row r="61">
@@ -1395,7 +1395,7 @@
         <v>4233489.4</v>
       </c>
       <c r="D61" t="n">
-        <v>30440752.43</v>
+        <v>16617185.7</v>
       </c>
     </row>
     <row r="62">
@@ -1411,7 +1411,7 @@
         <v>4182391.48</v>
       </c>
       <c r="D62" t="n">
-        <v>28686558.04</v>
+        <v>16264905.64</v>
       </c>
     </row>
     <row r="63">
@@ -1427,7 +1427,7 @@
         <v>2893966.57</v>
       </c>
       <c r="D63" t="n">
-        <v>24728075.43</v>
+        <v>13309888.59</v>
       </c>
     </row>
     <row r="64">
@@ -1443,7 +1443,7 @@
         <v>2657290.88</v>
       </c>
       <c r="D64" t="n">
-        <v>20411521.36</v>
+        <v>10929612.81</v>
       </c>
     </row>
     <row r="65">
@@ -1459,7 +1459,7 @@
         <v>2316504.14</v>
       </c>
       <c r="D65" t="n">
-        <v>17893656.29</v>
+        <v>9577518.109999999</v>
       </c>
     </row>
     <row r="66">
@@ -1475,7 +1475,7 @@
         <v>1046753.96</v>
       </c>
       <c r="D66" t="n">
-        <v>6627608.41</v>
+        <v>3726032.09</v>
       </c>
     </row>
     <row r="67">
@@ -1491,7 +1491,7 @@
         <v>500578.12</v>
       </c>
       <c r="D67" t="n">
-        <v>4067969.31</v>
+        <v>2146491.04</v>
       </c>
     </row>
     <row r="68">
@@ -1507,7 +1507,7 @@
         <v>437755.41</v>
       </c>
       <c r="D68" t="n">
-        <v>2916177.36</v>
+        <v>1629085.1</v>
       </c>
     </row>
     <row r="69">
@@ -1523,7 +1523,7 @@
         <v>262156.21</v>
       </c>
       <c r="D69" t="n">
-        <v>2060152.92</v>
+        <v>1095640.88</v>
       </c>
     </row>
     <row r="70">
@@ -1539,7 +1539,7 @@
         <v>179800.31</v>
       </c>
       <c r="D70" t="n">
-        <v>1176942.54</v>
+        <v>660001.85</v>
       </c>
     </row>
     <row r="71">
@@ -1555,7 +1555,7 @@
         <v>172883.32</v>
       </c>
       <c r="D71" t="n">
-        <v>1137355.23</v>
+        <v>637137.2</v>
       </c>
     </row>
     <row r="72">
@@ -1571,7 +1571,7 @@
         <v>86880.42</v>
       </c>
       <c r="D72" t="n">
-        <v>669990.29</v>
+        <v>358451.48</v>
       </c>
     </row>
     <row r="73">
@@ -1587,7 +1587,7 @@
         <v>34604.71</v>
       </c>
       <c r="D73" t="n">
-        <v>268062.93</v>
+        <v>143208.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza saídas com regra ContAgil (col E, +1 dia).
Reprocessa 2009–2010 com capitalização a partir do dia seguinte à parcela.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_por_agente.xlsx
+++ b/output/resumo_por_agente.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,129 +441,1153 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BANCO SANTANDER BRASIL SA</t>
+          <t>BANCO DO BRASIL SA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>42113</v>
       </c>
       <c r="C2" t="n">
-        <v>278419.45</v>
+        <v>5341100463.42</v>
       </c>
       <c r="D2" t="n">
-        <v>1020721.29</v>
+        <v>19592705069</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BANCO BRADESCO SA</t>
+          <t>ITAU UNIBANCO S.A.</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>56467</v>
       </c>
       <c r="C3" t="n">
-        <v>194561.72</v>
+        <v>4135945773.13</v>
       </c>
       <c r="D3" t="n">
-        <v>748057.86</v>
+        <v>15919764179.13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL SA</t>
+          <t>BANCO BRADESCO S.A.</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>56957</v>
       </c>
       <c r="C4" t="n">
-        <v>171859.57</v>
+        <v>3633054899.21</v>
       </c>
       <c r="D4" t="n">
-        <v>713232.4300000001</v>
+        <v>14115772612.38</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ITAU UNIBANCO SA</t>
+          <t>BANCO VOLKSWAGEN S.A.</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>50036</v>
       </c>
       <c r="C5" t="n">
-        <v>169963.48</v>
+        <v>1296591623.5</v>
       </c>
       <c r="D5" t="n">
-        <v>667455.28</v>
+        <v>5275760744.04</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
+          <t>BANCO SANTANDER (BRASIL) S.A.</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>13238</v>
       </c>
       <c r="C6" t="n">
-        <v>45846.49</v>
+        <v>1084182486.84</v>
       </c>
       <c r="D6" t="n">
-        <v>177713.77</v>
+        <v>4335172915.47</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO SICREDI SA</t>
+          <t>BANCO MERCEDES-BENZ DO BRASIL S/A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>22681</v>
       </c>
       <c r="C7" t="n">
-        <v>25504.66</v>
+        <v>1014242948.99</v>
       </c>
       <c r="D7" t="n">
-        <v>111238.29</v>
+        <v>4138151390.42</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAIXA ECONOMICA FEDERAL</t>
+          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>8402</v>
       </c>
       <c r="C8" t="n">
-        <v>19432.36</v>
+        <v>984715144.34</v>
       </c>
       <c r="D8" t="n">
-        <v>81482.09</v>
+        <v>3565677844.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO DO BRASIL SA - BANCOOB</t>
+          <t>BANCO SAFRA S A</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>12463</v>
+      </c>
+      <c r="C9" t="n">
+        <v>809780070.38</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3222977718.91</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BANCO VOTORANTIM S.A.</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4316</v>
+      </c>
+      <c r="C10" t="n">
+        <v>761998368.98</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2949641240.98</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KIRTON BANK S.A. - BANCO MULTIPLO</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3130</v>
+      </c>
+      <c r="C11" t="n">
+        <v>388257303.01</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1567405585.38</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BANCO CATERPILLAR S.A.</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4783</v>
+      </c>
+      <c r="C12" t="n">
+        <v>386132093.14</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1540860494.82</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BANCO ABC BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C13" t="n">
+        <v>346296018.75</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1378921846.72</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BANCO VOLVO (BRASIL) S.A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5818</v>
+      </c>
+      <c r="C14" t="n">
+        <v>299018659.68</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1192905704.21</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CAIXA ECONOMICA FEDERAL</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5071</v>
+      </c>
+      <c r="C15" t="n">
+        <v>278237123.01</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1075878902.47</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICREDI S.A.</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>12554</v>
+      </c>
+      <c r="C16" t="n">
+        <v>273580750.27</v>
+      </c>
+      <c r="D16" t="n">
+        <v>995400282.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A. - BDMG</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>631</v>
+      </c>
+      <c r="C17" t="n">
+        <v>225065011.59</v>
+      </c>
+      <c r="D17" t="n">
+        <v>817966395.78</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BADESUL DESENVOLVIMENTO S.A. - AGENCIA DE FOMENTO/RS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>968</v>
+      </c>
+      <c r="C18" t="n">
+        <v>221513408.22</v>
+      </c>
+      <c r="D18" t="n">
+        <v>805902261.83</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BANCO STELLANTIS S.A.</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4554</v>
+      </c>
+      <c r="C19" t="n">
+        <v>172291920.22</v>
+      </c>
+      <c r="D19" t="n">
+        <v>691341640.85</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DO RIO GRANDE DO SUL SA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3542</v>
+      </c>
+      <c r="C20" t="n">
+        <v>162181525.97</v>
+      </c>
+      <c r="D20" t="n">
+        <v>604754943.87</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BANCO PINE S/A</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>145</v>
+      </c>
+      <c r="C21" t="n">
+        <v>146127004.91</v>
+      </c>
+      <c r="D21" t="n">
+        <v>525418587.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BANCO DE LAGE LANDEN BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1214</v>
+      </c>
+      <c r="C22" t="n">
+        <v>121523832.93</v>
+      </c>
+      <c r="D22" t="n">
+        <v>472193094.97</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DO ESPIRITO SANTO S/A</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5011</v>
+      </c>
+      <c r="C23" t="n">
+        <v>100638150.52</v>
+      </c>
+      <c r="D23" t="n">
+        <v>358612642.34</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BANCO MONEO S.A.</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1177</v>
+      </c>
+      <c r="C24" t="n">
+        <v>93618588.05</v>
+      </c>
+      <c r="D24" t="n">
+        <v>369895885.44</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO COM INTERACAO SOLIDARIA</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8118</v>
+      </c>
+      <c r="C25" t="n">
+        <v>90357570.64</v>
+      </c>
+      <c r="D25" t="n">
+        <v>341570994.44</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO E ECONOMIA COM INTERACAO</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>6909</v>
+      </c>
+      <c r="C26" t="n">
+        <v>83013175.06999999</v>
+      </c>
+      <c r="D26" t="n">
+        <v>312435002.83</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SAFRA LEASING S.A. ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C27" t="n">
+        <v>72939004.75</v>
+      </c>
+      <c r="D27" t="n">
+        <v>305241620.22</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BANCO DA AMAZONIA SA / FINAM</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>41</v>
+      </c>
+      <c r="C28" t="n">
+        <v>71672467.09</v>
+      </c>
+      <c r="D28" t="n">
+        <v>253993844.25</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BANCO CNH INDUSTRIAL CAPITAL S.A.</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1154</v>
+      </c>
+      <c r="C29" t="n">
+        <v>68871369.95999999</v>
+      </c>
+      <c r="D29" t="n">
+        <v>281069691.29</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BANCO ALFA DE INVESTIMENTO S.A.</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>337</v>
+      </c>
+      <c r="C30" t="n">
+        <v>64836074.46</v>
+      </c>
+      <c r="D30" t="n">
+        <v>254902148.03</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICOOB S.A.</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>4244</v>
+      </c>
+      <c r="C31" t="n">
+        <v>56960724.06</v>
+      </c>
+      <c r="D31" t="n">
+        <v>211124714.7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BANCO DAYCOVAL S.A.</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>408</v>
+      </c>
+      <c r="C32" t="n">
+        <v>54878861.17</v>
+      </c>
+      <c r="D32" t="n">
+        <v>216531238.04</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BANCO RODOBENS S.A.</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2380</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51294982.03</v>
+      </c>
+      <c r="D33" t="n">
+        <v>209728098.11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BRADESCO LEASING S.A. - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>844</v>
+      </c>
+      <c r="C34" t="n">
+        <v>49858498.58</v>
+      </c>
+      <c r="D34" t="n">
+        <v>200394119.73</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BANCO DO NORDESTE DO BRASIL SA / FINOR</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>752</v>
+      </c>
+      <c r="C35" t="n">
+        <v>44547311.64</v>
+      </c>
+      <c r="D35" t="n">
+        <v>152782765.88</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BANCO FIBRA SA</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>292</v>
+      </c>
+      <c r="C36" t="n">
+        <v>42638582.93</v>
+      </c>
+      <c r="D36" t="n">
+        <v>184210051.14</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BANCO CITIBANK S A</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>320</v>
+      </c>
+      <c r="C37" t="n">
+        <v>40990391.88</v>
+      </c>
+      <c r="D37" t="n">
+        <v>165106650.13</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BANCO GUANABARA S/A</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>807</v>
+      </c>
+      <c r="C38" t="n">
+        <v>33621577.15</v>
+      </c>
+      <c r="D38" t="n">
+        <v>139540938.81</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SCANIA BANCO S.A.</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>395</v>
+      </c>
+      <c r="C39" t="n">
+        <v>31925061.26</v>
+      </c>
+      <c r="D39" t="n">
+        <v>120451676.85</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BANCO JOHN DEERE S.A.</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>374</v>
+      </c>
+      <c r="C40" t="n">
+        <v>31572895.34</v>
+      </c>
+      <c r="D40" t="n">
+        <v>123026119.36</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FINANCEIRA ALFA S.A. CREDITO, FINANCIAMENTO E INVESTIME</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>275</v>
+      </c>
+      <c r="C41" t="n">
+        <v>30442890.41</v>
+      </c>
+      <c r="D41" t="n">
+        <v>126646851.94</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MERCEDES-BENZ LEASING DO BRASIL ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>910</v>
+      </c>
+      <c r="C42" t="n">
+        <v>29331080.64</v>
+      </c>
+      <c r="D42" t="n">
+        <v>123644824.78</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BANESTES SA BANCO DO ESTADO DO ESPIRITO SANTO</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>144</v>
+      </c>
+      <c r="C43" t="n">
+        <v>21782951.19</v>
+      </c>
+      <c r="D43" t="n">
+        <v>86760013.22</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DE SANTA CATARINA S.A. - B</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>104</v>
+      </c>
+      <c r="C44" t="n">
+        <v>19116806.88</v>
+      </c>
+      <c r="D44" t="n">
+        <v>76518973.59999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BANCO RENDIMENTO S/A</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>84</v>
+      </c>
+      <c r="C45" t="n">
+        <v>17390467.3</v>
+      </c>
+      <c r="D45" t="n">
+        <v>69407776.61</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DESENVOLVE SP AGENCIA DE FOMENTO DO ESTADO DE SAO PAULO</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>214</v>
+      </c>
+      <c r="C46" t="n">
+        <v>16734761.99</v>
+      </c>
+      <c r="D46" t="n">
+        <v>67693251.97</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BANCO RIBEIRAO PRETO S/A</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>76</v>
+      </c>
+      <c r="C47" t="n">
+        <v>16278109.7</v>
+      </c>
+      <c r="D47" t="n">
+        <v>67514401.78</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BANCO VOITER SA</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>95</v>
+      </c>
+      <c r="C48" t="n">
+        <v>14018314.94</v>
+      </c>
+      <c r="D48" t="n">
+        <v>59493015.2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BANCO ITAULEASING S.A.</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>271</v>
+      </c>
+      <c r="C49" t="n">
+        <v>12785896.61</v>
+      </c>
+      <c r="D49" t="n">
+        <v>50827383.49</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BANCO BMG S.A</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>232</v>
+      </c>
+      <c r="C50" t="n">
+        <v>12405399.05</v>
+      </c>
+      <c r="D50" t="n">
+        <v>51279904.68</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO AMAZONAS S.A. - AFEAM</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>13</v>
+      </c>
+      <c r="C51" t="n">
+        <v>10963860.48</v>
+      </c>
+      <c r="D51" t="n">
+        <v>39928910.02</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BANCO RABOBANK INTERNATIONAL BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>39</v>
+      </c>
+      <c r="C52" t="n">
+        <v>10641060.28</v>
+      </c>
+      <c r="D52" t="n">
+        <v>38811838.33</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BRB BANCO DE BRASILIA SA</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>23</v>
+      </c>
+      <c r="C53" t="n">
+        <v>9241117.17</v>
+      </c>
+      <c r="D53" t="n">
+        <v>35578294.75</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BANCO INDUSTRIAL DO BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>107</v>
+      </c>
+      <c r="C54" t="n">
+        <v>9014630.560000001</v>
+      </c>
+      <c r="D54" t="n">
+        <v>37173490.49</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DIBENS LEASING S/A - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>112</v>
+      </c>
+      <c r="C55" t="n">
+        <v>8975145.720000001</v>
+      </c>
+      <c r="D55" t="n">
+        <v>37815729.98</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BANCO J. SAFRA S.A</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>85</v>
+      </c>
+      <c r="C56" t="n">
+        <v>6205254.78</v>
+      </c>
+      <c r="D56" t="n">
+        <v>27283686.64</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO RIO DE JANEIRO S. A.</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>18</v>
+      </c>
+      <c r="C57" t="n">
+        <v>5987175.05</v>
+      </c>
+      <c r="D57" t="n">
+        <v>23441394.09</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BANCO SOFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>62</v>
+      </c>
+      <c r="C58" t="n">
+        <v>5818096.47</v>
+      </c>
+      <c r="D58" t="n">
+        <v>26365698.98</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DE SERGIPE S/A</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>22</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4830549.81</v>
+      </c>
+      <c r="D59" t="n">
+        <v>17300875.48</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BANCO BTG PACTUAL S.A.</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>14</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4535918.69</v>
+      </c>
+      <c r="D60" t="n">
+        <v>18580937.51</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BANCO TRIANGULO S/A</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>43</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4233489.4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>16612858.43</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DESENBAHIA-AGENCIA DE FOMENTO DO ESTADO DA BAHIA S/A</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>29</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4182391.48</v>
+      </c>
+      <c r="D62" t="n">
+        <v>16260759</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BANCO CREFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>25</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2893966.57</v>
+      </c>
+      <c r="D63" t="n">
+        <v>13306621.94</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BANCO BV S.A.</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>40</v>
+      </c>
+      <c r="C64" t="n">
+        <v>2657290.88</v>
+      </c>
+      <c r="D64" t="n">
+        <v>10926855.12</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BMG LEASING SA ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>41</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2316504.14</v>
+      </c>
+      <c r="D65" t="n">
+        <v>9575057.92</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BB.LEASING S.A.ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>17</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1046753.96</v>
+      </c>
+      <c r="D66" t="n">
+        <v>3725036.16</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BRKB DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS S.A</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="n">
-        <v>6319.76</v>
-      </c>
-      <c r="D9" t="n">
-        <v>26013.92</v>
+      <c r="C67" t="n">
+        <v>500578.12</v>
+      </c>
+      <c r="D67" t="n">
+        <v>2145949.13</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BANCO RANDON SA</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="n">
+        <v>437755.41</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1628650.82</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DIRECAO S A CREDITO FINANCIAMENTO E INVESTIMENTO</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>6</v>
+      </c>
+      <c r="C69" t="n">
+        <v>262156.21</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1095364.9</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO PARANA S.A.</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="n">
+        <v>179800.31</v>
+      </c>
+      <c r="D70" t="n">
+        <v>659828.65</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO TOCANTINS S.A.</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" t="n">
+        <v>172883.32</v>
+      </c>
+      <c r="D71" t="n">
+        <v>636969.98</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BANCO PORTO REAL DE INVESTIMENTOS S/A</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>86880.42</v>
+      </c>
+      <c r="D72" t="n">
+        <v>358362.99</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BONCRED FINANCEIRA S.A. - CREDITO, FINANCIAMENTO E INVE</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" t="n">
+        <v>34604.71</v>
+      </c>
+      <c r="D73" t="n">
+        <v>143173.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementa lógica corrigida de fluxos ContAgil (dual balance + taxa efetiva).
Adiciona taxa_contrato_efetiva (TAXA FIXA / TJLP/TLP), saldos fiscal e de
contrato, subsídio pré-amortização e atualiza testes e saídas de amostra.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_por_agente.xlsx
+++ b/output/resumo_por_agente.xlsx
@@ -441,65 +441,65 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BANCO SANTANDER BRASIL SA</t>
+          <t>BANCO DO BRASIL SA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>278419.45</v>
+        <v>171859.57</v>
       </c>
       <c r="D2" t="n">
-        <v>1020721.29</v>
+        <v>1338244.62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BANCO BRADESCO SA</t>
+          <t>BANCO SANTANDER BRASIL SA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>194561.72</v>
+        <v>145344.49</v>
       </c>
       <c r="D3" t="n">
-        <v>748057.86</v>
+        <v>951850.9300000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BANCO DO BRASIL SA</t>
+          <t>ITAU UNIBANCO SA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>171859.57</v>
+        <v>112878.86</v>
       </c>
       <c r="D4" t="n">
-        <v>713232.4300000001</v>
+        <v>785962.01</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ITAU UNIBANCO SA</t>
+          <t>BANCO BRADESCO SA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>169963.48</v>
+        <v>81317.25999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>667455.28</v>
+        <v>579838.11</v>
       </c>
     </row>
     <row r="6">
@@ -515,7 +515,7 @@
         <v>45846.49</v>
       </c>
       <c r="D6" t="n">
-        <v>177713.77</v>
+        <v>323583.93</v>
       </c>
     </row>
     <row r="7">
@@ -531,7 +531,7 @@
         <v>25504.66</v>
       </c>
       <c r="D7" t="n">
-        <v>111238.29</v>
+        <v>212271.05</v>
       </c>
     </row>
     <row r="8">
@@ -547,7 +547,7 @@
         <v>19432.36</v>
       </c>
       <c r="D8" t="n">
-        <v>81482.09</v>
+        <v>153424.44</v>
       </c>
     </row>
     <row r="9">
@@ -563,7 +563,7 @@
         <v>6319.76</v>
       </c>
       <c r="D9" t="n">
-        <v>26013.92</v>
+        <v>48575.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish ContAgil --full run results for 2009–2010 BNDES.
348,864 contracts / 22.15M parcels; subsidy R$21.41bi; impact R$81.59bi
with corrected dual-balance logic and Bacen SELIC factors.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_por_agente.xlsx
+++ b/output/resumo_por_agente.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,125 +445,1149 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>42113</v>
       </c>
       <c r="C2" t="n">
-        <v>171859.57</v>
+        <v>4994115924.23</v>
       </c>
       <c r="D2" t="n">
-        <v>1338244.62</v>
+        <v>18179058533.54</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BANCO SANTANDER BRASIL SA</t>
+          <t>ITAU UNIBANCO S.A.</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>56467</v>
       </c>
       <c r="C3" t="n">
-        <v>145344.49</v>
+        <v>3830977062.56</v>
       </c>
       <c r="D3" t="n">
-        <v>951850.9300000001</v>
+        <v>14630913781.65</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ITAU UNIBANCO SA</t>
+          <t>BANCO BRADESCO S.A.</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>56957</v>
       </c>
       <c r="C4" t="n">
-        <v>112878.86</v>
+        <v>3342969848.59</v>
       </c>
       <c r="D4" t="n">
-        <v>785962.01</v>
+        <v>12852176710.82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BANCO BRADESCO SA</t>
+          <t>BANCO VOLKSWAGEN S.A.</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>50036</v>
       </c>
       <c r="C5" t="n">
-        <v>81317.25999999999</v>
+        <v>1106086892.95</v>
       </c>
       <c r="D5" t="n">
-        <v>579838.11</v>
+        <v>4448982244.03</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
+          <t>BANCO SANTANDER (BRASIL) S.A.</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>13238</v>
       </c>
       <c r="C6" t="n">
-        <v>45846.49</v>
+        <v>961158838.8200001</v>
       </c>
       <c r="D6" t="n">
-        <v>323583.93</v>
+        <v>3807098515.86</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO SICREDI SA</t>
+          <t>BANCO REGIONAL DE DESENVOLVIMENTO DO EXTREMO SUL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>8402</v>
       </c>
       <c r="C7" t="n">
-        <v>25504.66</v>
+        <v>858220103.53</v>
       </c>
       <c r="D7" t="n">
-        <v>212271.05</v>
+        <v>3107947362.74</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAIXA ECONOMICA FEDERAL</t>
+          <t>BANCO MERCEDES-BENZ DO BRASIL S/A</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>22681</v>
       </c>
       <c r="C8" t="n">
-        <v>19432.36</v>
+        <v>813261397.25</v>
       </c>
       <c r="D8" t="n">
-        <v>153424.44</v>
+        <v>3269634957.03</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BANCO COOPERATIVO DO BRASIL SA - BANCOOB</t>
+          <t>BANCO SAFRA S A</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>12463</v>
+      </c>
+      <c r="C9" t="n">
+        <v>773081172.54</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3066369279.75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BANCO VOTORANTIM S.A.</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4316</v>
+      </c>
+      <c r="C10" t="n">
+        <v>703574792.8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2715088172.08</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>KIRTON BANK S.A. - BANCO MULTIPLO</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3130</v>
+      </c>
+      <c r="C11" t="n">
+        <v>355708719.88</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1430917914.11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BANCO CATERPILLAR S.A.</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4783</v>
+      </c>
+      <c r="C12" t="n">
+        <v>348478104.94</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1373191228.25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BANCO ABC BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C13" t="n">
+        <v>329864204.53</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1307564035.66</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BANCO VOLVO (BRASIL) S.A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5818</v>
+      </c>
+      <c r="C14" t="n">
+        <v>272472851.61</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1077009932.84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICREDI S.A.</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>12554</v>
+      </c>
+      <c r="C15" t="n">
+        <v>270059277.48</v>
+      </c>
+      <c r="D15" t="n">
+        <v>981257101.63</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CAIXA ECONOMICA FEDERAL</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5071</v>
+      </c>
+      <c r="C16" t="n">
+        <v>238858951.27</v>
+      </c>
+      <c r="D16" t="n">
+        <v>910734869.41</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A. - BDMG</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>631</v>
+      </c>
+      <c r="C17" t="n">
+        <v>192687508.78</v>
+      </c>
+      <c r="D17" t="n">
+        <v>689618078.9400001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BADESUL DESENVOLVIMENTO S.A. - AGENCIA DE FOMENTO/RS</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>968</v>
+      </c>
+      <c r="C18" t="n">
+        <v>192032488.18</v>
+      </c>
+      <c r="D18" t="n">
+        <v>690301472.28</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BANCO STELLANTIS S.A.</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4554</v>
+      </c>
+      <c r="C19" t="n">
+        <v>150854227.63</v>
+      </c>
+      <c r="D19" t="n">
+        <v>598506270.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BANCO PINE S/A</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>145</v>
+      </c>
+      <c r="C20" t="n">
+        <v>146127004.91</v>
+      </c>
+      <c r="D20" t="n">
+        <v>525418587.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DO RIO GRANDE DO SUL SA</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3542</v>
+      </c>
+      <c r="C21" t="n">
+        <v>145366117.63</v>
+      </c>
+      <c r="D21" t="n">
+        <v>533593693.96</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BANCO DE LAGE LANDEN BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1214</v>
+      </c>
+      <c r="C22" t="n">
+        <v>116842823.37</v>
+      </c>
+      <c r="D22" t="n">
+        <v>451862471.61</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BANCO DE DESENVOLVIMENTO DO ESPIRITO SANTO S/A</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5011</v>
+      </c>
+      <c r="C23" t="n">
+        <v>97851569.47</v>
+      </c>
+      <c r="D23" t="n">
+        <v>347657883.74</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO COM INTERACAO SOLIDARIA</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8118</v>
+      </c>
+      <c r="C24" t="n">
+        <v>90292636.75</v>
+      </c>
+      <c r="D24" t="n">
+        <v>341298523.02</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COOPERATIVA CENTRAL DE CREDITO E ECONOMIA COM INTERACAO</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6909</v>
+      </c>
+      <c r="C25" t="n">
+        <v>82894836.58</v>
+      </c>
+      <c r="D25" t="n">
+        <v>311947806.25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BANCO MONEO S.A.</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1177</v>
+      </c>
+      <c r="C26" t="n">
+        <v>77239194.5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>301315481.33</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SAFRA LEASING S.A. ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C27" t="n">
+        <v>72939004.75</v>
+      </c>
+      <c r="D27" t="n">
+        <v>305241620.22</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BANCO DA AMAZONIA SA / FINAM</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>41</v>
+      </c>
+      <c r="C28" t="n">
+        <v>68144073.34</v>
+      </c>
+      <c r="D28" t="n">
+        <v>240074256.92</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BANCO DAYCOVAL S.A.</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>408</v>
+      </c>
+      <c r="C29" t="n">
+        <v>54627816.48</v>
+      </c>
+      <c r="D29" t="n">
+        <v>215456100.67</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BANCO COOPERATIVO SICOOB S.A.</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4244</v>
+      </c>
+      <c r="C30" t="n">
+        <v>54319046.1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>200403418.28</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BANCO CNH INDUSTRIAL CAPITAL S.A.</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1154</v>
+      </c>
+      <c r="C31" t="n">
+        <v>54028040.12</v>
+      </c>
+      <c r="D31" t="n">
+        <v>216313023.97</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BANCO ALFA DE INVESTIMENTO S.A.</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>337</v>
+      </c>
+      <c r="C32" t="n">
+        <v>50750139.92</v>
+      </c>
+      <c r="D32" t="n">
+        <v>196665082.54</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BRADESCO LEASING S.A. - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>844</v>
+      </c>
+      <c r="C33" t="n">
+        <v>49858498.58</v>
+      </c>
+      <c r="D33" t="n">
+        <v>200394119.73</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BANCO DO NORDESTE DO BRASIL SA / FINOR</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>752</v>
+      </c>
+      <c r="C34" t="n">
+        <v>44227984.86</v>
+      </c>
+      <c r="D34" t="n">
+        <v>151427577.87</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BANCO RODOBENS S.A.</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2380</v>
+      </c>
+      <c r="C35" t="n">
+        <v>43213797.26</v>
+      </c>
+      <c r="D35" t="n">
+        <v>174582873.38</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BANCO FIBRA SA</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>292</v>
+      </c>
+      <c r="C36" t="n">
+        <v>41710748.33</v>
+      </c>
+      <c r="D36" t="n">
+        <v>180179581.51</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BANCO CITIBANK S A</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>320</v>
+      </c>
+      <c r="C37" t="n">
+        <v>39221773.16</v>
+      </c>
+      <c r="D37" t="n">
+        <v>157344666.47</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SCANIA BANCO S.A.</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>395</v>
+      </c>
+      <c r="C38" t="n">
+        <v>31925061.26</v>
+      </c>
+      <c r="D38" t="n">
+        <v>120451676.85</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BANCO GUANABARA S/A</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>807</v>
+      </c>
+      <c r="C39" t="n">
+        <v>30874389.29</v>
+      </c>
+      <c r="D39" t="n">
+        <v>127011072.82</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BANCO JOHN DEERE S.A.</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>374</v>
+      </c>
+      <c r="C40" t="n">
+        <v>30233579.65</v>
+      </c>
+      <c r="D40" t="n">
+        <v>117285023.51</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MERCEDES-BENZ LEASING DO BRASIL ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>910</v>
+      </c>
+      <c r="C41" t="n">
+        <v>29331080.64</v>
+      </c>
+      <c r="D41" t="n">
+        <v>123644824.78</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>FINANCEIRA ALFA S.A. CREDITO, FINANCIAMENTO E INVESTIME</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>275</v>
+      </c>
+      <c r="C42" t="n">
+        <v>21439921.62</v>
+      </c>
+      <c r="D42" t="n">
+        <v>87382146.56</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BANESTES SA BANCO DO ESTADO DO ESPIRITO SANTO</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>144</v>
+      </c>
+      <c r="C43" t="n">
+        <v>18665959.34</v>
+      </c>
+      <c r="D43" t="n">
+        <v>73174626.31999999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BANCO RENDIMENTO S/A</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>84</v>
+      </c>
+      <c r="C44" t="n">
+        <v>16832026.79</v>
+      </c>
+      <c r="D44" t="n">
+        <v>67092918.08</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DESENVOLVE SP AGENCIA DE FOMENTO DO ESTADO DE SAO PAULO</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>214</v>
+      </c>
+      <c r="C45" t="n">
+        <v>16552079.34</v>
+      </c>
+      <c r="D45" t="n">
+        <v>66997453.17</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BANCO RIBEIRAO PRETO S/A</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>76</v>
+      </c>
+      <c r="C46" t="n">
+        <v>14836633.76</v>
+      </c>
+      <c r="D46" t="n">
+        <v>61203854.52</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DE SANTA CATARINA S.A. - B</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>104</v>
+      </c>
+      <c r="C47" t="n">
+        <v>14237281.94</v>
+      </c>
+      <c r="D47" t="n">
+        <v>57455184.2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BANCO ITAULEASING S.A.</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>271</v>
+      </c>
+      <c r="C48" t="n">
+        <v>12785896.61</v>
+      </c>
+      <c r="D48" t="n">
+        <v>50827383.49</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BANCO VOITER SA</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>95</v>
+      </c>
+      <c r="C49" t="n">
+        <v>12434415.4</v>
+      </c>
+      <c r="D49" t="n">
+        <v>52501576.65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BANCO BMG S.A</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>232</v>
+      </c>
+      <c r="C50" t="n">
+        <v>12391908.37</v>
+      </c>
+      <c r="D50" t="n">
+        <v>51222962.97</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO AMAZONAS S.A. - AFEAM</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>13</v>
+      </c>
+      <c r="C51" t="n">
+        <v>10522300.45</v>
+      </c>
+      <c r="D51" t="n">
+        <v>38063815.51</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BANCO RABOBANK INTERNATIONAL BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>39</v>
+      </c>
+      <c r="C52" t="n">
+        <v>10237621.19</v>
+      </c>
+      <c r="D52" t="n">
+        <v>37271971.46</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DIBENS LEASING S/A - ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>112</v>
+      </c>
+      <c r="C53" t="n">
+        <v>8975145.720000001</v>
+      </c>
+      <c r="D53" t="n">
+        <v>37815729.98</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BANCO INDUSTRIAL DO BRASIL S/A</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>107</v>
+      </c>
+      <c r="C54" t="n">
+        <v>8629098.640000001</v>
+      </c>
+      <c r="D54" t="n">
+        <v>35484755.83</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BRB BANCO DE BRASILIA SA</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>23</v>
+      </c>
+      <c r="C55" t="n">
+        <v>7895590.19</v>
+      </c>
+      <c r="D55" t="n">
+        <v>30307259.02</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO RIO DE JANEIRO S. A.</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>18</v>
+      </c>
+      <c r="C56" t="n">
+        <v>5987175.05</v>
+      </c>
+      <c r="D56" t="n">
+        <v>23441394.09</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BANCO DO ESTADO DE SERGIPE S/A</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>22</v>
+      </c>
+      <c r="C57" t="n">
+        <v>4830549.81</v>
+      </c>
+      <c r="D57" t="n">
+        <v>17300875.48</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BANCO SOFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>62</v>
+      </c>
+      <c r="C58" t="n">
+        <v>4605471.88</v>
+      </c>
+      <c r="D58" t="n">
+        <v>21439370.33</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BANCO BTG PACTUAL S.A.</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>14</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4535918.69</v>
+      </c>
+      <c r="D59" t="n">
+        <v>18580937.51</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DESENBAHIA-AGENCIA DE FOMENTO DO ESTADO DA BAHIA S/A</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>29</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4182391.48</v>
+      </c>
+      <c r="D60" t="n">
+        <v>16260759</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BANCO TRIANGULO S/A</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>43</v>
+      </c>
+      <c r="C61" t="n">
+        <v>3510309.55</v>
+      </c>
+      <c r="D61" t="n">
+        <v>13900927.84</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BANCO J. SAFRA S.A</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>85</v>
+      </c>
+      <c r="C62" t="n">
+        <v>2724822.39</v>
+      </c>
+      <c r="D62" t="n">
+        <v>11965655.93</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BANCO BV S.A.</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>40</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2657290.88</v>
+      </c>
+      <c r="D63" t="n">
+        <v>10926855.12</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BANCO CREFISA S.A.</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>25</v>
+      </c>
+      <c r="C64" t="n">
+        <v>2497187.71</v>
+      </c>
+      <c r="D64" t="n">
+        <v>11478986.19</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BMG LEASING SA ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>41</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2316504.14</v>
+      </c>
+      <c r="D65" t="n">
+        <v>9575057.92</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BB.LEASING S.A.ARRENDAMENTO MERCANTIL</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>17</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1046753.96</v>
+      </c>
+      <c r="D66" t="n">
+        <v>3725036.16</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BRKB DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS S.A</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
         <v>1</v>
       </c>
-      <c r="C9" t="n">
-        <v>6319.76</v>
-      </c>
-      <c r="D9" t="n">
-        <v>48575.92</v>
+      <c r="C67" t="n">
+        <v>500578.12</v>
+      </c>
+      <c r="D67" t="n">
+        <v>2145949.13</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BANCO RANDON SA</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="n">
+        <v>437755.41</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1628650.82</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DIRECAO S A CREDITO FINANCIAMENTO E INVESTIMENTO</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>6</v>
+      </c>
+      <c r="C69" t="n">
+        <v>226474.14</v>
+      </c>
+      <c r="D69" t="n">
+        <v>935227.8199999999</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO ESTADO DO TOCANTINS S.A.</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>5</v>
+      </c>
+      <c r="C70" t="n">
+        <v>172883.32</v>
+      </c>
+      <c r="D70" t="n">
+        <v>636969.98</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>AGENCIA DE FOMENTO DO PARANA S.A.</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>4</v>
+      </c>
+      <c r="C71" t="n">
+        <v>130972.11</v>
+      </c>
+      <c r="D71" t="n">
+        <v>479312.14</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BANCO PORTO REAL DE INVESTIMENTOS S/A</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>86880.42</v>
+      </c>
+      <c r="D72" t="n">
+        <v>358362.99</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BONCRED FINANCEIRA S.A. - CREDITO, FINANCIAMENTO E INVE</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" t="n">
+        <v>-10264.94</v>
+      </c>
+      <c r="D73" t="n">
+        <v>98044.39999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>